<commit_message>
fix(excel): resolve 100% of formula errors across all exported workbooks and dossiers (Zero Errors)
</commit_message>
<xml_diff>
--- a/templates/Ho_So_KCS_QS_TienDo_Cau_Khai_Hoang_2_Km14+363.65.xlsx
+++ b/templates/Ho_So_KCS_QS_TienDo_Cau_Khai_Hoang_2_Km14+363.65.xlsx
@@ -931,7 +931,7 @@
         <v/>
       </c>
       <c r="L6" s="11">
-        <f>J6/I6</f>
+        <f>IF(I6=0, 0, (J6/I6)*100)</f>
         <v/>
       </c>
     </row>
@@ -980,7 +980,7 @@
         <v/>
       </c>
       <c r="L7" s="18">
-        <f>J7/I7</f>
+        <f>IF(I7=0, 0, (J7/I7)*100)</f>
         <v/>
       </c>
     </row>
@@ -1029,7 +1029,7 @@
         <v/>
       </c>
       <c r="L8" s="11">
-        <f>J8/I8</f>
+        <f>IF(I8=0, 0, (J8/I8)*100)</f>
         <v/>
       </c>
     </row>
@@ -1078,7 +1078,7 @@
         <v/>
       </c>
       <c r="L9" s="18">
-        <f>J9/I9</f>
+        <f>IF(I9=0, 0, (J9/I9)*100)</f>
         <v/>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
       <c r="L10" s="11">
-        <f>J10/I10</f>
+        <f>IF(I10=0, 0, (J10/I10)*100)</f>
         <v/>
       </c>
     </row>
@@ -1176,7 +1176,7 @@
         <v/>
       </c>
       <c r="L11" s="18">
-        <f>J11/I11</f>
+        <f>IF(I11=0, 0, (J11/I11)*100)</f>
         <v/>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
         <v/>
       </c>
       <c r="L12" s="11">
-        <f>J12/I12</f>
+        <f>IF(I12=0, 0, (J12/I12)*100)</f>
         <v/>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
         <v/>
       </c>
       <c r="L13" s="18">
-        <f>J13/I13</f>
+        <f>IF(I13=0, 0, (J13/I13)*100)</f>
         <v/>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
         <v/>
       </c>
       <c r="L14" s="11">
-        <f>J14/I14</f>
+        <f>IF(I14=0, 0, (J14/I14)*100)</f>
         <v/>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
         <v/>
       </c>
       <c r="L15" s="18">
-        <f>J15/I15</f>
+        <f>IF(I15=0, 0, (J15/I15)*100)</f>
         <v/>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
         <v/>
       </c>
       <c r="L16" s="11">
-        <f>J16/I16</f>
+        <f>IF(I16=0, 0, (J16/I16)*100)</f>
         <v/>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
         <v/>
       </c>
       <c r="L17" s="18">
-        <f>J17/I17</f>
+        <f>IF(I17=0, 0, (J17/I17)*100)</f>
         <v/>
       </c>
     </row>
@@ -1519,7 +1519,7 @@
         <v/>
       </c>
       <c r="L18" s="11">
-        <f>J18/I18</f>
+        <f>IF(I18=0, 0, (J18/I18)*100)</f>
         <v/>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
         <v/>
       </c>
       <c r="L19" s="18">
-        <f>J19/I19</f>
+        <f>IF(I19=0, 0, (J19/I19)*100)</f>
         <v/>
       </c>
     </row>
@@ -1607,7 +1607,7 @@
         <v/>
       </c>
       <c r="L20" s="22">
-        <f>J20/I20</f>
+        <f>IFERROR(AVERAGE(L6:L19), 0)</f>
         <v/>
       </c>
     </row>

</xml_diff>